<commit_message>
Set up initial graph with Chart.js
</commit_message>
<xml_diff>
--- a/public/CareerOneStop_Data.xlsx
+++ b/public/CareerOneStop_Data.xlsx
@@ -7,7 +7,7 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +22,7 @@
     <t>Occupation</t>
   </si>
   <si>
-    <t>2022 Employment</t>
+    <t>2022 NJ Employment</t>
   </si>
   <si>
     <t>Earnings</t>
@@ -49,10 +49,10 @@
     <t>Fastest_Growing_Rank</t>
   </si>
   <si>
-    <t>2024 Employment</t>
-  </si>
-  <si>
-    <t>2034 Employment</t>
+    <t>2024 US Employment</t>
+  </si>
+  <si>
+    <t>2034 US Employment</t>
   </si>
   <si>
     <t>Percent Change</t>

</xml_diff>